<commit_message>
feat: enhance postal code extraction and normalization
- Added support for English names of provinces, districts, and subdistricts in the extraction process.
- Introduced slug style options for generating slugs in various formats (e.g., slug-case, snake_case, camelCase).
- Updated the CLI to accept new options for slug style and English column names.
- Modified the normalization process to include English names and generate slugs based on the selected style.
- Enhanced database schema and output formats to accommodate new fields for English names.
- Updated tests to verify the extraction and normalization of English names and slug generation.
</commit_message>
<xml_diff>
--- a/test/fixtures/postal-codes.fixture.xlsx
+++ b/test/fixtures/postal-codes.fixture.xlsx
@@ -4,15 +4,19 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Source" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Postal" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="WorksheetFallback" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="TambonDatabase" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="35">
+  <si>
+    <t>TambonID</t>
+  </si>
   <si>
     <t>ตำบล</t>
   </si>
@@ -56,9 +60,6 @@
     <t>PostCode</t>
   </si>
   <si>
-    <t>TambonID</t>
-  </si>
-  <si>
     <t>หมายเหตุ</t>
   </si>
   <si>
@@ -81,6 +82,42 @@
   </si>
   <si>
     <t>สัมพันธวงศ์</t>
+  </si>
+  <si>
+    <t>TambonEngShort</t>
+  </si>
+  <si>
+    <t>DistrictEngShort</t>
+  </si>
+  <si>
+    <t>ProvinceEng</t>
+  </si>
+  <si>
+    <t>Phra Borom Maha Ratchawang</t>
+  </si>
+  <si>
+    <t>Phra Nakhon</t>
+  </si>
+  <si>
+    <t>Bangkok</t>
+  </si>
+  <si>
+    <t>Si Phum</t>
+  </si>
+  <si>
+    <t>Mueang Chiang Mai</t>
+  </si>
+  <si>
+    <t>เชียงใหม่</t>
+  </si>
+  <si>
+    <t>Chiang Mai</t>
+  </si>
+  <si>
+    <t>Chakkrawat</t>
+  </si>
+  <si>
+    <t>Samphanthawong</t>
   </si>
 </sst>
 </file>
@@ -136,18 +173,20 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="รหัสไปรษณีย์" displayName="รหัสไปรษณีย์" ref="A1:D4" totalsRowShown="1" headerRowCount="1">
-  <autoFilter ref="A1:D4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="รหัสไปรษณีย์" displayName="รหัสไปรษณีย์" ref="A1:E4" totalsRowShown="1" headerRowCount="1">
+  <autoFilter ref="A1:E4">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
     <filterColumn colId="3" hiddenButton="1"/>
+    <filterColumn colId="4" hiddenButton="1"/>
   </autoFilter>
-  <tableColumns count="4">
-    <tableColumn id="1" name="ตำบล" totalsRowLabel="Total"/>
-    <tableColumn id="2" name="อำเภอ" totalsRowFunction="none"/>
-    <tableColumn id="3" name="จังหวัด" totalsRowFunction="none"/>
-    <tableColumn id="4" name="รหัสไปรษณีย์" totalsRowFunction="none"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="TambonID" totalsRowLabel="Total"/>
+    <tableColumn id="2" name="ตำบล" totalsRowFunction="none"/>
+    <tableColumn id="3" name="อำเภอ" totalsRowFunction="none"/>
+    <tableColumn id="4" name="จังหวัด" totalsRowFunction="none"/>
+    <tableColumn id="5" name="รหัสไปรษณีย์" totalsRowFunction="none"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -170,6 +209,30 @@
     <tableColumn id="4" name="TambonThaiShort" totalsRowFunction="none"/>
     <tableColumn id="5" name="DistrictThaiShort" totalsRowFunction="none"/>
     <tableColumn id="6" name="ProvinceThai" totalsRowFunction="none"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" name="ThepExcelTambon" displayName="ThepExcelTambon" ref="A1:G4" totalsRowShown="1" headerRowCount="1">
+  <autoFilter ref="A1:G4">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
+    <filterColumn colId="4" hiddenButton="1"/>
+    <filterColumn colId="5" hiddenButton="1"/>
+    <filterColumn colId="6" hiddenButton="1"/>
+  </autoFilter>
+  <tableColumns count="7">
+    <tableColumn id="1" name="TambonID" totalsRowLabel="Total"/>
+    <tableColumn id="2" name="TambonThaiShort" totalsRowFunction="none"/>
+    <tableColumn id="3" name="TambonEngShort" totalsRowFunction="none"/>
+    <tableColumn id="4" name="DistrictThaiShort" totalsRowFunction="none"/>
+    <tableColumn id="5" name="DistrictEngShort" totalsRowFunction="none"/>
+    <tableColumn id="6" name="ProvinceThai" totalsRowFunction="none"/>
+    <tableColumn id="7" name="ProvinceEng" totalsRowFunction="none"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -497,10 +560,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -513,10 +576,13 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="E1" t="s">
         <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>100101</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
@@ -524,27 +590,33 @@
       <c r="C2" t="s">
         <v>6</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2">
         <v>10200</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>7</v>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>100101</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
       </c>
       <c r="D3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" t="s">
         <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>500101</v>
       </c>
       <c r="B4" t="s">
         <v>10</v>
@@ -555,10 +627,13 @@
       <c r="D4" t="s">
         <v>12</v>
       </c>
+      <c r="E4" t="s">
+        <v>13</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
@@ -572,10 +647,10 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B1" t="s">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="C1" t="s">
         <v>15</v>
@@ -604,7 +679,113 @@
         <v>22</v>
       </c>
       <c r="F2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" t="s">
+        <v>24</v>
+      </c>
+      <c r="F1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>100101</v>
+      </c>
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" t="s">
         <v>6</v>
+      </c>
+      <c r="E2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>500101</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>101301</v>
+      </c>
+      <c r="B4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>